<commit_message>
Sửa lỗi phân quyền chỉnh sửa, phê duyệt, gởi email cho quản lý
</commit_message>
<xml_diff>
--- a/cung_cap_dl/kho_bao_tri/bao_tri/danh_sach_nm.xlsx
+++ b/cung_cap_dl/kho_bao_tri/bao_tri/danh_sach_nm.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Software\rubber-erp\cung_cap_dl\kho_bao_tri\bao_tri\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{35C0B8B5-7C57-484F-AD4A-DF6D56D7C333}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{07B34663-653D-4795-AF50-65969E488885}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -170,7 +170,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="6" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="10"/>
       <color rgb="FF000000"/>
@@ -202,23 +202,6 @@
       <charset val="163"/>
       <scheme val="major"/>
     </font>
-    <font>
-      <u/>
-      <sz val="10"/>
-      <color theme="10"/>
-      <name val="Arial"/>
-      <family val="2"/>
-      <charset val="163"/>
-      <scheme val="major"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF000000"/>
-      <name val="Arial"/>
-      <family val="2"/>
-      <charset val="163"/>
-      <scheme val="major"/>
-    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -241,22 +224,21 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="14" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="14" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="14" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="14" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -483,11 +465,11 @@
   <dimension ref="A1:F15"/>
   <sheetFormatPr defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="12.6640625" style="3"/>
-    <col min="2" max="2" width="31.6640625" style="3" customWidth="1"/>
-    <col min="3" max="3" width="23.77734375" style="3" customWidth="1"/>
-    <col min="4" max="4" width="31.21875" style="3" customWidth="1"/>
-    <col min="5" max="6" width="12.6640625" style="3"/>
+    <col min="1" max="1" width="12.6640625" style="2"/>
+    <col min="2" max="2" width="31.6640625" style="2" customWidth="1"/>
+    <col min="3" max="3" width="23.77734375" style="2" customWidth="1"/>
+    <col min="4" max="4" width="31.21875" style="2" customWidth="1"/>
+    <col min="5" max="6" width="12.6640625" style="2"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="13.2" x14ac:dyDescent="0.25">
@@ -517,10 +499,10 @@
       <c r="C2" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="D2" s="4" t="s">
+      <c r="D2" s="6" t="s">
         <v>40</v>
       </c>
-      <c r="E2" s="5">
+      <c r="E2" s="3">
         <v>32465</v>
       </c>
     </row>
@@ -534,10 +516,10 @@
       <c r="C3" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="D3" s="6" t="s">
+      <c r="D3" s="5" t="s">
         <v>44</v>
       </c>
-      <c r="E3" s="7">
+      <c r="E3" s="4">
         <v>34398</v>
       </c>
     </row>
@@ -551,14 +533,14 @@
       <c r="C4" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="D4" s="6" t="s">
+      <c r="D4" s="5" t="s">
         <v>41</v>
       </c>
-      <c r="E4" s="7">
+      <c r="E4" s="4">
         <v>36586</v>
       </c>
     </row>
-    <row r="5" spans="1:5" ht="13.8" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:5" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
         <v>11</v>
       </c>
@@ -568,10 +550,9 @@
       <c r="C5" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="D5" s="8" t="s">
+      <c r="D5" s="7" t="s">
         <v>46</v>
       </c>
-      <c r="E5" s="2"/>
     </row>
     <row r="6" spans="1:5" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
@@ -583,10 +564,10 @@
       <c r="C6" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="D6" s="6" t="s">
+      <c r="D6" s="5" t="s">
         <v>42</v>
       </c>
-      <c r="E6" s="7">
+      <c r="E6" s="4">
         <v>36931</v>
       </c>
     </row>
@@ -600,10 +581,10 @@
       <c r="C7" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="D7" s="6" t="s">
+      <c r="D7" s="5" t="s">
         <v>43</v>
       </c>
-      <c r="E7" s="7">
+      <c r="E7" s="4">
         <v>37173</v>
       </c>
     </row>
@@ -617,8 +598,6 @@
       <c r="C8" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="D8" s="2"/>
-      <c r="E8" s="2"/>
     </row>
     <row r="9" spans="1:5" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A9" s="1" t="s">
@@ -630,8 +609,6 @@
       <c r="C9" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="D9" s="2"/>
-      <c r="E9" s="2"/>
     </row>
     <row r="10" spans="1:5" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A10" s="1" t="s">
@@ -643,8 +620,6 @@
       <c r="C10" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="D10" s="2"/>
-      <c r="E10" s="2"/>
     </row>
     <row r="11" spans="1:5" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A11" s="1" t="s">
@@ -656,8 +631,6 @@
       <c r="C11" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="D11" s="2"/>
-      <c r="E11" s="2"/>
     </row>
     <row r="12" spans="1:5" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A12" s="1" t="s">
@@ -669,8 +642,6 @@
       <c r="C12" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="D12" s="2"/>
-      <c r="E12" s="2"/>
     </row>
     <row r="13" spans="1:5" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A13" s="1" t="s">
@@ -682,8 +653,6 @@
       <c r="C13" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="D13" s="2"/>
-      <c r="E13" s="2"/>
     </row>
     <row r="14" spans="1:5" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A14" s="1" t="s">
@@ -695,8 +664,6 @@
       <c r="C14" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="D14" s="2"/>
-      <c r="E14" s="2"/>
     </row>
     <row r="15" spans="1:5" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A15" s="1" t="s">
@@ -708,12 +675,15 @@
       <c r="C15" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="D15" s="2"/>
-      <c r="E15" s="2"/>
     </row>
   </sheetData>
   <hyperlinks>
     <hyperlink ref="D2" r:id="rId1" xr:uid="{ED104ED8-F4D7-452B-8A5F-B82A9D95693C}"/>
+    <hyperlink ref="D4" r:id="rId2" xr:uid="{9733A346-97AE-4094-9B65-021077634DC8}"/>
+    <hyperlink ref="D3" r:id="rId3" xr:uid="{8FE4D329-65F9-46D0-AE7D-8747A0B46A0C}"/>
+    <hyperlink ref="D7" r:id="rId4" xr:uid="{66A6DDC3-8050-4FD8-9F46-444C13378855}"/>
+    <hyperlink ref="D6" r:id="rId5" xr:uid="{1BC9408F-B928-4087-AE28-9587DEF519B1}"/>
+    <hyperlink ref="D5" r:id="rId6" xr:uid="{84491440-AC42-4C23-B3F9-27D3B86FD65F}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>